<commit_message>
Rename Provincia España to Total
</commit_message>
<xml_diff>
--- a/data/processed/university_dimensions.xlsx
+++ b/data/processed/university_dimensions.xlsx
@@ -1805,7 +1805,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">

</xml_diff>